<commit_message>
Correct under-$200 picks against full placement history
Client's month-by-month placement history revealed heavy overlap with the
vendor list; rebuilt exclusion set (727 domains) and re-filtered. Removed
already-built picks (kitchenfunwithmy3sons, roadfood, retail-insider,
chefs-resources, fb101, awesomecuisine, mykitchenstories, intheplayroom,
etc.). Final list is truly not-built, non-alcohol, relevant, under $200.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EyZhZSnP6QyNR5y5EJdqhU
</commit_message>
<xml_diff>
--- a/nangwizard-under200-picks.xlsx
+++ b/nangwizard-under200-picks.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Under $200 (Semrush metrics)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Not-built &lt;$200 (Semrush)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,17 +423,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BUY (branded anchor)</t>
+          <t>BUY (AU, branded anchor)</t>
         </is>
       </c>
     </row>
@@ -545,28 +545,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kitchenfunwithmy3sons.com</t>
+          <t>live-less-ordinary.com</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>English: Family Recipes, Dinner Ideas, Desserts &amp; Ba</t>
+          <t>English: Travel, Food &amp; Drink, Lifestyle</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
-        <v>257330</v>
+        <v>155532</v>
       </c>
       <c r="F4" t="n">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="G4" t="n">
-        <v>8328</v>
+        <v>2399</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -577,28 +577,28 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>retail-insider.com</t>
+          <t>conservamome.com</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Retail News, Industry Insights, News, Food</t>
+          <t>English: Parenting, Recipes, Lifestyle, Crafts, Fa</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D5" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>39291</v>
+        <v>37485</v>
       </c>
       <c r="F5" t="n">
-        <v>190</v>
+        <v>130</v>
       </c>
       <c r="G5" t="n">
-        <v>7095</v>
+        <v>2735</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -609,28 +609,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>conservamome.com</t>
+          <t>theworldonmynecklace.com</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>English: Parenting, Recipes, Lifestyle, Crafts, Fami</t>
+          <t>Travel, Adventure, Tips, Food, Destinations</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E6" t="n">
-        <v>37485</v>
+        <v>81024</v>
       </c>
       <c r="F6" t="n">
-        <v>130</v>
+        <v>175</v>
       </c>
       <c r="G6" t="n">
-        <v>2735</v>
+        <v>1077</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -641,28 +641,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>roadfood.com</t>
+          <t>gardenweb.com</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>English: Restaurants, Regional Cuisine, Food Travel,</t>
+          <t>English: Home &amp; garden forum, Kitchen &amp; dining ide</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D7" t="n">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="E7" t="n">
-        <v>34959</v>
+        <v>35244</v>
       </c>
       <c r="F7" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="G7" t="n">
-        <v>8226</v>
+        <v>12568</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -673,28 +673,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gardenweb.com</t>
+          <t>thesoulofseoul.net</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>English: Home &amp; garden forum, Kitchen &amp; dining ideas</t>
+          <t>English: Korea Travel, Seoul Guide, Culture, Food,</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>39</v>
       </c>
       <c r="D8" t="n">
-        <v>61</v>
+        <v>18</v>
       </c>
       <c r="E8" t="n">
-        <v>35244</v>
+        <v>113267</v>
       </c>
       <c r="F8" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="G8" t="n">
-        <v>12568</v>
+        <v>1803</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -705,28 +705,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>chefs-resources.com</t>
+          <t>traveltweaks.com</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Food &amp; Drink, Food, Recipes</t>
+          <t>Adventure, Airlines, Bar, Destinations, Events, Fo</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D9" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E9" t="n">
-        <v>52542</v>
+        <v>13406</v>
       </c>
       <c r="F9" t="n">
-        <v>182</v>
+        <v>90</v>
       </c>
       <c r="G9" t="n">
-        <v>2195</v>
+        <v>3775</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -737,28 +737,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>traveltweaks.com</t>
+          <t>pinoyadventurista.com</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Adventure, Airlines, Bar, Destinations, Events, Food</t>
+          <t>Adventure, Beaches, Blogs, English, Food, Food &amp; D</t>
         </is>
       </c>
       <c r="C10" t="n">
         <v>36</v>
       </c>
       <c r="D10" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E10" t="n">
-        <v>13406</v>
+        <v>55321</v>
       </c>
       <c r="F10" t="n">
-        <v>90</v>
+        <v>180</v>
       </c>
       <c r="G10" t="n">
-        <v>3775</v>
+        <v>2119</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -769,60 +769,60 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>live-less-ordinary.com</t>
+          <t>artsreview.com.au</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>English: Travel, Food &amp; Drink, Lifestyle</t>
+          <t>Arts &amp; Entertainment, Entertainment, Culture, Revi</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="D11" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E11" t="n">
-        <v>155532</v>
+        <v>11706</v>
       </c>
       <c r="F11" t="n">
-        <v>150</v>
+        <v>186</v>
       </c>
       <c r="G11" t="n">
-        <v>2399</v>
+        <v>2288</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>BUY (AU)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>theworldonmynecklace.com</t>
+          <t>beontheroad.com</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Travel, Adventure, Tips, Food, Destinations</t>
+          <t>Travel, Adventure, Food, Lifestyle</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D12" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E12" t="n">
-        <v>81024</v>
+        <v>32581</v>
       </c>
       <c r="F12" t="n">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="G12" t="n">
-        <v>1077</v>
+        <v>782</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -833,28 +833,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>intheplayroom.co.uk</t>
+          <t>orangewayfarer.com</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Breastfeedingguide, Craft, Diyresources, English, En</t>
+          <t>English: Travel Blog, Cultural Travel Stories, Foo</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D13" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E13" t="n">
-        <v>20965</v>
+        <v>32811</v>
       </c>
       <c r="F13" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G13" t="n">
-        <v>5275</v>
+        <v>645</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -865,92 +865,92 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>awesomecuisine.com</t>
+          <t>emmysmummy.com</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Food &amp; Drink, Food, Recipes</t>
+          <t>English: Parenting &amp; family life, Lifestyle, Trave</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D14" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E14" t="n">
-        <v>19902</v>
+        <v>4321</v>
       </c>
       <c r="F14" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="G14" t="n">
-        <v>3080</v>
+        <v>1045</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Secondary (family)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>artsreview.com.au</t>
+          <t>sweetlivingmagazine.co.nz</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arts &amp; Entertainment, Entertainment, Culture, Review</t>
+          <t>Home &amp; Garden, Home, Decor</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D15" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>11706</v>
+        <v>11368</v>
       </c>
       <c r="F15" t="n">
-        <v>186</v>
+        <v>144</v>
       </c>
       <c r="G15" t="n">
-        <v>2288</v>
+        <v>888</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Secondary (AU)</t>
+          <t>Secondary (NZ)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fb101.com</t>
+          <t>birdsandlilies.com</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Food, Blogging, Recipes</t>
+          <t>English: Lifestyle, Travel, Family, Health &amp; Fitne</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D16" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E16" t="n">
-        <v>8260</v>
+        <v>17660</v>
       </c>
       <c r="F16" t="n">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="G16" t="n">
-        <v>4500</v>
+        <v>798</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -961,32 +961,160 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>mykitchenstories.com.au</t>
+          <t>rachelbustin.com</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>English: Food &amp; Drink, Lifestyle, Home Cooking</t>
+          <t xml:space="preserve">English: Parenting, Family life, Product reviews, </t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D17" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E17" t="n">
-        <v>25777</v>
+        <v>4120</v>
       </c>
       <c r="F17" t="n">
-        <v>150</v>
+        <v>98</v>
       </c>
       <c r="G17" t="n">
-        <v>800</v>
+        <v>1216</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Secondary (AU)</t>
+          <t>Secondary (family)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>brightonsavoy.com.au</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Weddings, Events, Accommodation</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>30</v>
+      </c>
+      <c r="D18" t="n">
+        <v>23</v>
+      </c>
+      <c r="E18" t="n">
+        <v>11332</v>
+      </c>
+      <c r="F18" t="n">
+        <v>145</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2003</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Secondary (AU/Melbourne)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>placesandfoods.com</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Travelling, Travel, Tourism, Food</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>29</v>
+      </c>
+      <c r="D19" t="n">
+        <v>21</v>
+      </c>
+      <c r="E19" t="n">
+        <v>14966</v>
+      </c>
+      <c r="F19" t="n">
+        <v>126</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2807</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Secondary</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ourkidsmom.com</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>English: Parenting, Family lifestyle, Recipes, Tra</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>29</v>
+      </c>
+      <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" t="n">
+        <v>5918</v>
+      </c>
+      <c r="F20" t="n">
+        <v>120</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2445</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Secondary (family)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>whatkatysaid.com</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Parenting, Lifestyle, Recipes, Home</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>29</v>
+      </c>
+      <c r="D21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4375</v>
+      </c>
+      <c r="F21" t="n">
+        <v>190</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1335</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Secondary (family)</t>
         </is>
       </c>
     </row>

</xml_diff>